<commit_message>
Files are refactored for the new shotgunSurgerySmell.py
</commit_message>
<xml_diff>
--- a/util/Analysis/BadSmells/ShotgunSurgery/ShotgunSurgerySmellRelationAnalysisOfkeras.xlsx
+++ b/util/Analysis/BadSmells/ShotgunSurgery/ShotgunSurgerySmellRelationAnalysisOfkeras.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11010"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neda/Documents/workspace/DissertationProject/util/Analysis/BadSmells/ShotgunSurgery/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neda/Documents/PycharmProjects/DissertationProject/util/Analysis/BadSmells/ShotgunSurgery/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EBCF95D5-7EEC-4D43-BB42-6F89088E9CB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{914DA1BD-B6F6-414B-8107-16FFDE4ABDA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="460" windowWidth="25440" windowHeight="14000"/>
+    <workbookView xWindow="80" yWindow="460" windowWidth="25440" windowHeight="14000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ShotgunSurgerySmellRelationAnal" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ShotgunSurgerySmellRelationAnal!$A$1:$I$270</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -625,7 +628,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -1459,7 +1462,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I270"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -1492,7 +1496,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1521,7 +1525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1550,7 +1554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -1579,7 +1583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1608,7 +1612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1637,7 +1641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -1666,7 +1670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>13</v>
       </c>
@@ -1695,7 +1699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -1724,7 +1728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -1753,7 +1757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1782,7 +1786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1811,7 +1815,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -1840,7 +1844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -1869,7 +1873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1898,7 +1902,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -1927,7 +1931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -1956,7 +1960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -1985,7 +1989,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>23</v>
       </c>
@@ -2014,7 +2018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>24</v>
       </c>
@@ -2043,7 +2047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>25</v>
       </c>
@@ -2072,7 +2076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>26</v>
       </c>
@@ -2101,7 +2105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -2130,7 +2134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>28</v>
       </c>
@@ -2159,7 +2163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>29</v>
       </c>
@@ -2188,7 +2192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -2217,7 +2221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>31</v>
       </c>
@@ -2246,7 +2250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>32</v>
       </c>
@@ -2275,7 +2279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>33</v>
       </c>
@@ -2304,7 +2308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>34</v>
       </c>
@@ -2333,7 +2337,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>35</v>
       </c>
@@ -2478,7 +2482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>42</v>
       </c>
@@ -2507,7 +2511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>43</v>
       </c>
@@ -2536,7 +2540,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>43</v>
       </c>
@@ -2565,7 +2569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>43</v>
       </c>
@@ -2594,7 +2598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>44</v>
       </c>
@@ -2623,7 +2627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>45</v>
       </c>
@@ -2652,7 +2656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>46</v>
       </c>
@@ -2681,7 +2685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>47</v>
       </c>
@@ -2710,7 +2714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -2739,7 +2743,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>49</v>
       </c>
@@ -2768,7 +2772,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>50</v>
       </c>
@@ -2797,7 +2801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>51</v>
       </c>
@@ -2826,7 +2830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>52</v>
       </c>
@@ -2855,7 +2859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>53</v>
       </c>
@@ -2884,7 +2888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>54</v>
       </c>
@@ -2913,7 +2917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>55</v>
       </c>
@@ -2942,7 +2946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>56</v>
       </c>
@@ -2971,7 +2975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>56</v>
       </c>
@@ -3000,7 +3004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>57</v>
       </c>
@@ -3029,7 +3033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>58</v>
       </c>
@@ -3058,7 +3062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>59</v>
       </c>
@@ -3087,7 +3091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>60</v>
       </c>
@@ -3116,7 +3120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>61</v>
       </c>
@@ -3145,7 +3149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>62</v>
       </c>
@@ -3174,7 +3178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>63</v>
       </c>
@@ -3203,7 +3207,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>64</v>
       </c>
@@ -3232,7 +3236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>65</v>
       </c>
@@ -3261,7 +3265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>66</v>
       </c>
@@ -3290,7 +3294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>67</v>
       </c>
@@ -3319,7 +3323,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>68</v>
       </c>
@@ -3348,7 +3352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>69</v>
       </c>
@@ -3377,7 +3381,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>70</v>
       </c>
@@ -3406,7 +3410,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>71</v>
       </c>
@@ -3435,7 +3439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>72</v>
       </c>
@@ -3464,7 +3468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>72</v>
       </c>
@@ -3493,7 +3497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>46</v>
       </c>
@@ -3522,7 +3526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>46</v>
       </c>
@@ -3551,7 +3555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>47</v>
       </c>
@@ -3580,7 +3584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>47</v>
       </c>
@@ -3609,7 +3613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>73</v>
       </c>
@@ -3638,7 +3642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>74</v>
       </c>
@@ -3667,7 +3671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>75</v>
       </c>
@@ -3696,7 +3700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>76</v>
       </c>
@@ -3725,7 +3729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>77</v>
       </c>
@@ -3754,7 +3758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>78</v>
       </c>
@@ -3783,7 +3787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>79</v>
       </c>
@@ -3812,7 +3816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>80</v>
       </c>
@@ -3841,7 +3845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>81</v>
       </c>
@@ -3870,7 +3874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>82</v>
       </c>
@@ -3899,7 +3903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>83</v>
       </c>
@@ -3928,7 +3932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>84</v>
       </c>
@@ -3957,7 +3961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>85</v>
       </c>
@@ -3986,7 +3990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>86</v>
       </c>
@@ -4015,7 +4019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>87</v>
       </c>
@@ -4044,7 +4048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>88</v>
       </c>
@@ -4073,7 +4077,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>89</v>
       </c>
@@ -4102,7 +4106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>90</v>
       </c>
@@ -4131,7 +4135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>91</v>
       </c>
@@ -4160,7 +4164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>92</v>
       </c>
@@ -4189,7 +4193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>93</v>
       </c>
@@ -4218,7 +4222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>94</v>
       </c>
@@ -4247,7 +4251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>95</v>
       </c>
@@ -4276,7 +4280,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>96</v>
       </c>
@@ -4305,7 +4309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>97</v>
       </c>
@@ -4334,7 +4338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>98</v>
       </c>
@@ -4363,7 +4367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>99</v>
       </c>
@@ -4392,7 +4396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>100</v>
       </c>
@@ -4421,7 +4425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>101</v>
       </c>
@@ -4450,7 +4454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>102</v>
       </c>
@@ -4479,7 +4483,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>103</v>
       </c>
@@ -4508,7 +4512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>104</v>
       </c>
@@ -4537,7 +4541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>105</v>
       </c>
@@ -4566,7 +4570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>106</v>
       </c>
@@ -4595,7 +4599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>106</v>
       </c>
@@ -4624,7 +4628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>107</v>
       </c>
@@ -4653,7 +4657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>108</v>
       </c>
@@ -4682,7 +4686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>108</v>
       </c>
@@ -4711,7 +4715,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>109</v>
       </c>
@@ -4740,7 +4744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>110</v>
       </c>
@@ -4769,7 +4773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>110</v>
       </c>
@@ -4798,7 +4802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>111</v>
       </c>
@@ -4827,7 +4831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>112</v>
       </c>
@@ -4856,7 +4860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>112</v>
       </c>
@@ -4885,7 +4889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>113</v>
       </c>
@@ -4914,7 +4918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>114</v>
       </c>
@@ -4943,7 +4947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>114</v>
       </c>
@@ -4972,7 +4976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>115</v>
       </c>
@@ -5001,7 +5005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>116</v>
       </c>
@@ -5030,7 +5034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>116</v>
       </c>
@@ -5059,7 +5063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>117</v>
       </c>
@@ -5088,7 +5092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>56</v>
       </c>
@@ -5117,7 +5121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>118</v>
       </c>
@@ -5146,7 +5150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>118</v>
       </c>
@@ -5175,7 +5179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>119</v>
       </c>
@@ -5204,7 +5208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>119</v>
       </c>
@@ -5233,7 +5237,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>120</v>
       </c>
@@ -5262,7 +5266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>121</v>
       </c>
@@ -5291,7 +5295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>122</v>
       </c>
@@ -5320,7 +5324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>123</v>
       </c>
@@ -5349,7 +5353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>124</v>
       </c>
@@ -5378,7 +5382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>125</v>
       </c>
@@ -5407,7 +5411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>126</v>
       </c>
@@ -5436,7 +5440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>126</v>
       </c>
@@ -5465,7 +5469,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>127</v>
       </c>
@@ -5494,7 +5498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>128</v>
       </c>
@@ -5523,7 +5527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>129</v>
       </c>
@@ -5552,7 +5556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>130</v>
       </c>
@@ -5581,7 +5585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>130</v>
       </c>
@@ -5610,7 +5614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>131</v>
       </c>
@@ -5639,7 +5643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>132</v>
       </c>
@@ -5668,7 +5672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>133</v>
       </c>
@@ -5697,7 +5701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>134</v>
       </c>
@@ -5726,7 +5730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>135</v>
       </c>
@@ -5755,7 +5759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>136</v>
       </c>
@@ -5784,7 +5788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>136</v>
       </c>
@@ -5813,7 +5817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>137</v>
       </c>
@@ -5842,7 +5846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>137</v>
       </c>
@@ -5871,7 +5875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>138</v>
       </c>
@@ -5900,7 +5904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>138</v>
       </c>
@@ -5929,7 +5933,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>139</v>
       </c>
@@ -5958,7 +5962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>140</v>
       </c>
@@ -5987,7 +5991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>141</v>
       </c>
@@ -6016,7 +6020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>142</v>
       </c>
@@ -6045,7 +6049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>143</v>
       </c>
@@ -6074,7 +6078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>144</v>
       </c>
@@ -6103,7 +6107,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>145</v>
       </c>
@@ -6132,7 +6136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>146</v>
       </c>
@@ -6161,7 +6165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>147</v>
       </c>
@@ -6190,7 +6194,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>148</v>
       </c>
@@ -6219,7 +6223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>149</v>
       </c>
@@ -6248,7 +6252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>150</v>
       </c>
@@ -6277,7 +6281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>40</v>
       </c>
@@ -6306,7 +6310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>40</v>
       </c>
@@ -6335,7 +6339,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>40</v>
       </c>
@@ -6364,7 +6368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>12</v>
       </c>
@@ -6393,7 +6397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>12</v>
       </c>
@@ -6422,7 +6426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>12</v>
       </c>
@@ -6451,7 +6455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>12</v>
       </c>
@@ -6480,7 +6484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>12</v>
       </c>
@@ -6509,7 +6513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>12</v>
       </c>
@@ -6538,7 +6542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>12</v>
       </c>
@@ -6567,7 +6571,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>61</v>
       </c>
@@ -6596,7 +6600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>22</v>
       </c>
@@ -6625,7 +6629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>22</v>
       </c>
@@ -6654,7 +6658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>22</v>
       </c>
@@ -6683,7 +6687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>151</v>
       </c>
@@ -6712,7 +6716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>152</v>
       </c>
@@ -6741,7 +6745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>152</v>
       </c>
@@ -6770,7 +6774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>153</v>
       </c>
@@ -6799,7 +6803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>154</v>
       </c>
@@ -6828,7 +6832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>45</v>
       </c>
@@ -6857,7 +6861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>48</v>
       </c>
@@ -6886,7 +6890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>49</v>
       </c>
@@ -6915,7 +6919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>50</v>
       </c>
@@ -6944,7 +6948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>51</v>
       </c>
@@ -6973,7 +6977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>52</v>
       </c>
@@ -7002,7 +7006,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>155</v>
       </c>
@@ -7031,7 +7035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>9</v>
       </c>
@@ -7060,7 +7064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>156</v>
       </c>
@@ -7089,7 +7093,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>157</v>
       </c>
@@ -7118,7 +7122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>157</v>
       </c>
@@ -7147,7 +7151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>158</v>
       </c>
@@ -7176,7 +7180,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>158</v>
       </c>
@@ -7205,7 +7209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>159</v>
       </c>
@@ -7234,7 +7238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>160</v>
       </c>
@@ -7263,7 +7267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>161</v>
       </c>
@@ -7292,7 +7296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>151</v>
       </c>
@@ -7321,7 +7325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>152</v>
       </c>
@@ -7350,7 +7354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>62</v>
       </c>
@@ -7379,7 +7383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>62</v>
       </c>
@@ -7408,7 +7412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>162</v>
       </c>
@@ -7437,7 +7441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>163</v>
       </c>
@@ -7466,7 +7470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>164</v>
       </c>
@@ -7495,7 +7499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>165</v>
       </c>
@@ -7524,7 +7528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>12</v>
       </c>
@@ -7553,7 +7557,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>166</v>
       </c>
@@ -7582,7 +7586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>167</v>
       </c>
@@ -7611,7 +7615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>168</v>
       </c>
@@ -7640,7 +7644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>169</v>
       </c>
@@ -7843,7 +7847,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>35</v>
       </c>
@@ -7872,7 +7876,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>35</v>
       </c>
@@ -7901,7 +7905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>9</v>
       </c>
@@ -7930,7 +7934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>177</v>
       </c>
@@ -7959,7 +7963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>178</v>
       </c>
@@ -7988,7 +7992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>62</v>
       </c>
@@ -8017,7 +8021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>165</v>
       </c>
@@ -8046,7 +8050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>13</v>
       </c>
@@ -8075,7 +8079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>13</v>
       </c>
@@ -8104,7 +8108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>13</v>
       </c>
@@ -8133,7 +8137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>179</v>
       </c>
@@ -8162,7 +8166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>180</v>
       </c>
@@ -8191,7 +8195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>181</v>
       </c>
@@ -8220,7 +8224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>182</v>
       </c>
@@ -8249,7 +8253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>183</v>
       </c>
@@ -8278,7 +8282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>184</v>
       </c>
@@ -8307,7 +8311,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>19</v>
       </c>
@@ -8336,7 +8340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>21</v>
       </c>
@@ -8365,7 +8369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>23</v>
       </c>
@@ -8394,7 +8398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="240" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>23</v>
       </c>
@@ -8423,7 +8427,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="241" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>26</v>
       </c>
@@ -8452,7 +8456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>27</v>
       </c>
@@ -8481,7 +8485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>28</v>
       </c>
@@ -8510,7 +8514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="244" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>29</v>
       </c>
@@ -8539,7 +8543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>30</v>
       </c>
@@ -8568,7 +8572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>31</v>
       </c>
@@ -8597,7 +8601,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>151</v>
       </c>
@@ -8626,7 +8630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>152</v>
       </c>
@@ -8655,7 +8659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>151</v>
       </c>
@@ -8684,7 +8688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>185</v>
       </c>
@@ -8713,7 +8717,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>186</v>
       </c>
@@ -8742,7 +8746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>187</v>
       </c>
@@ -8771,7 +8775,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>188</v>
       </c>
@@ -8800,7 +8804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>62</v>
       </c>
@@ -8829,7 +8833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>72</v>
       </c>
@@ -8858,7 +8862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>189</v>
       </c>
@@ -8887,7 +8891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>190</v>
       </c>
@@ -8916,7 +8920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>191</v>
       </c>
@@ -8945,7 +8949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>192</v>
       </c>
@@ -8974,7 +8978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>193</v>
       </c>
@@ -9003,7 +9007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
         <v>194</v>
       </c>
@@ -9032,7 +9036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
         <v>194</v>
       </c>
@@ -9061,7 +9065,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
         <v>195</v>
       </c>
@@ -9090,7 +9094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
         <v>196</v>
       </c>
@@ -9119,7 +9123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="265" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
         <v>197</v>
       </c>
@@ -9148,7 +9152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
         <v>198</v>
       </c>
@@ -9177,7 +9181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="267" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
         <v>68</v>
       </c>
@@ -9206,7 +9210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="268" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
         <v>22</v>
       </c>
@@ -9235,7 +9239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
         <v>22</v>
       </c>
@@ -9264,7 +9268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
         <v>199</v>
       </c>
@@ -9294,6 +9298,14 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:I270" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="2"/>
+        <filter val="3"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>